<commit_message>
Day 32: Implement capital allocation reporting and pattern analysis
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K98"/>
+  <dimension ref="A1:K93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4519,229 +4519,6 @@
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>UNITDSPR</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="C94" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>High Quality</t>
-        </is>
-      </c>
-      <c r="E94" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>Asset Light</t>
-        </is>
-      </c>
-      <c r="G94" t="n">
-        <v>22.91</v>
-      </c>
-      <c r="H94" t="n">
-        <v>63.67</v>
-      </c>
-      <c r="I94" t="b">
-        <v>0</v>
-      </c>
-      <c r="J94" t="b">
-        <v>0</v>
-      </c>
-      <c r="K94" t="inlineStr">
-        <is>
-          <t>Liquidating Assets</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>VEDL</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="C95" t="n">
-        <v>2.27</v>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>High Quality</t>
-        </is>
-      </c>
-      <c r="E95" t="n">
-        <v>9.470000000000001</v>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>Capital Intensive</t>
-        </is>
-      </c>
-      <c r="G95" t="n">
-        <v>13.22</v>
-      </c>
-      <c r="H95" t="n">
-        <v>59.28</v>
-      </c>
-      <c r="I95" t="b">
-        <v>0</v>
-      </c>
-      <c r="J95" t="b">
-        <v>1</v>
-      </c>
-      <c r="K95" t="inlineStr">
-        <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>WIPRO</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="C96" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>High Quality</t>
-        </is>
-      </c>
-      <c r="E96" t="n">
-        <v>1.29</v>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>Asset Light</t>
-        </is>
-      </c>
-      <c r="G96" t="n">
-        <v>8.27</v>
-      </c>
-      <c r="H96" t="n">
-        <v>105.59</v>
-      </c>
-      <c r="I96" t="b">
-        <v>0</v>
-      </c>
-      <c r="J96" t="b">
-        <v>0</v>
-      </c>
-      <c r="K96" t="inlineStr">
-        <is>
-          <t>Liquidating Assets</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>ZOMATO</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="C97" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="E97" t="n">
-        <v>1.94</v>
-      </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>Asset Light</t>
-        </is>
-      </c>
-      <c r="G97" t="inlineStr"/>
-      <c r="H97" t="n">
-        <v>45.78</v>
-      </c>
-      <c r="I97" t="b">
-        <v>0</v>
-      </c>
-      <c r="J97" t="b">
-        <v>0</v>
-      </c>
-      <c r="K97" t="inlineStr">
-        <is>
-          <t>Reinvestor</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>ZYDUSLIFE</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="C98" t="n">
-        <v>0.89</v>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="E98" t="n">
-        <v>6.94</v>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="G98" t="n">
-        <v>-2.59</v>
-      </c>
-      <c r="H98" t="n">
-        <v>27.65</v>
-      </c>
-      <c r="I98" t="b">
-        <v>0</v>
-      </c>
-      <c r="J98" t="b">
-        <v>1</v>
-      </c>
-      <c r="K98" t="inlineStr">
-        <is>
-          <t>Reinvestor</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>